<commit_message>
modified:   data/chapter2/FREDv3subset/state_conflicts.xlsx 	modified:   notebooks/chapter_02/populate_states.ipynb 	modified:   semseg/MaskRCNN/trial.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FREDv3subset/state_conflicts.xlsx
+++ b/data/chapter2/FREDv3subset/state_conflicts.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="305" documentId="11_F25DC773A252ABDACC1048FDB99E5A8E5BDE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C05750-F410-4D58-BB99-0B5249CBFA2A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="state_conflicts" sheetId="4" r:id="rId1"/>
@@ -580,8 +580,8 @@
   <autoFilter ref="A1:C68" xr:uid="{94A66970-29A1-4ABD-AEBE-D0A24611F563}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7D5055AE-5791-4C1F-A5D9-BD7F62E12A31}" name="binominal" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{CCCF8186-328A-492F-AF4E-343C0E157695}" name="actual_publication_reports_in_fungalroot" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{E697EBF1-06BD-4B49-AF8F-6BB250377B9E}" name="fungalroot_agreed_species_state" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{CCCF8186-328A-492F-AF4E-343C0E157695}" name="actual_publication_reports_in_fungalroot" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{E697EBF1-06BD-4B49-AF8F-6BB250377B9E}" name="fungalroot_agreed_species_state" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>